<commit_message>
Show completed semifinal standings in archive
</commit_message>
<xml_diff>
--- a/data/quotazioni/quotazioni_TERZOPOSTO.xlsx
+++ b/data/quotazioni/quotazioni_TERZOPOSTO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11116"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b9cb5207b7e2a247/Personale/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{1A118867-679C-0A49-BCF0-A0C981EA8BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71B9CF8D-D5B8-5742-AF5E-18C9AC408C01}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{1A118867-679C-0A49-BCF0-A0C981EA8BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDC382CF-F772-A24E-A294-4F713A045CCD}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -325,7 +325,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
@@ -338,6 +338,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -816,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -896,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -976,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -1056,7 +1060,7 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -1136,7 +1140,7 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1216,7 +1220,7 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1296,7 +1300,7 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -1376,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -1456,7 +1460,7 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -1536,7 +1540,7 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -1616,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -1696,7 +1700,7 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -1776,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -1856,7 +1860,7 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -1936,7 +1940,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -2016,7 +2020,7 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -2096,7 +2100,7 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -2176,7 +2180,7 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H20">
         <v>0</v>
@@ -2256,7 +2260,7 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H21">
         <v>0</v>
@@ -2336,7 +2340,7 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -2416,7 +2420,7 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -2496,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="G24">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H24">
         <v>0</v>
@@ -2576,7 +2580,7 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -2656,7 +2660,7 @@
         <v>0</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -2896,7 +2900,7 @@
         <v>0</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -2976,7 +2980,7 @@
         <v>0</v>
       </c>
       <c r="G30">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H30">
         <v>0</v>
@@ -3056,7 +3060,7 @@
         <v>0</v>
       </c>
       <c r="G31">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H31">
         <v>0</v>
@@ -3136,7 +3140,7 @@
         <v>0</v>
       </c>
       <c r="G32">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H32">
         <v>0</v>
@@ -3216,7 +3220,7 @@
         <v>0</v>
       </c>
       <c r="G33">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H33">
         <v>0</v>
@@ -3296,7 +3300,7 @@
         <v>0</v>
       </c>
       <c r="G34">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H34">
         <v>0</v>
@@ -3376,7 +3380,7 @@
         <v>0</v>
       </c>
       <c r="G35">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H35">
         <v>0</v>
@@ -3456,7 +3460,7 @@
         <v>0</v>
       </c>
       <c r="G36">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="H36">
         <v>0</v>
@@ -3536,7 +3540,7 @@
         <v>0</v>
       </c>
       <c r="G37">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="H37">
         <v>0</v>
@@ -3616,7 +3620,7 @@
         <v>0</v>
       </c>
       <c r="G38">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="H38">
         <v>0</v>
@@ -3696,7 +3700,7 @@
         <v>0</v>
       </c>
       <c r="G39">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="H39">
         <v>0</v>
@@ -3776,7 +3780,7 @@
         <v>0</v>
       </c>
       <c r="G40">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H40">
         <v>0</v>
@@ -3856,7 +3860,7 @@
         <v>0</v>
       </c>
       <c r="G41">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H41">
         <v>0</v>
@@ -3936,7 +3940,7 @@
         <v>0</v>
       </c>
       <c r="G42">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H42">
         <v>0</v>
@@ -4016,7 +4020,7 @@
         <v>0</v>
       </c>
       <c r="G43">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H43">
         <v>0</v>
@@ -4096,7 +4100,7 @@
         <v>0</v>
       </c>
       <c r="G44">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H44">
         <v>0</v>
@@ -4176,7 +4180,7 @@
         <v>0</v>
       </c>
       <c r="G45">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="H45">
         <v>0</v>
@@ -4256,7 +4260,7 @@
         <v>0</v>
       </c>
       <c r="G46">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H46">
         <v>0</v>
@@ -4336,7 +4340,7 @@
         <v>0</v>
       </c>
       <c r="G47">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H47">
         <v>0</v>
@@ -4416,7 +4420,7 @@
         <v>0</v>
       </c>
       <c r="G48">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H48">
         <v>0</v>
@@ -4496,7 +4500,7 @@
         <v>0</v>
       </c>
       <c r="G49">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H49">
         <v>0</v>
@@ -4576,7 +4580,7 @@
         <v>0</v>
       </c>
       <c r="G50">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H50">
         <v>0</v>
@@ -4656,7 +4660,7 @@
         <v>0</v>
       </c>
       <c r="G51">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H51">
         <v>0</v>
@@ -4736,7 +4740,7 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H52">
         <v>0</v>
@@ -4816,7 +4820,7 @@
         <v>0</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H53">
         <v>0</v>

</xml_diff>